<commit_message>
Add PiN by pop, step 1 hybrid  for Somalia___SOM
</commit_message>
<xml_diff>
--- a/platform_PiN_output/Somalia___SOM/PiN_pop_step1_Somalia___SOM_1008_02AM.xlsx
+++ b/platform_PiN_output/Somalia___SOM/PiN_pop_step1_Somalia___SOM_1008_02AM.xlsx
@@ -504,10 +504,10 @@
         <v>179099</v>
       </c>
       <c r="D2" t="n">
-        <v>60.7</v>
+        <v>60.4</v>
       </c>
       <c r="E2" t="n">
-        <v>108762</v>
+        <v>108111</v>
       </c>
       <c r="F2" t="n">
         <v>35.6</v>
@@ -522,16 +522,16 @@
         <v>5861</v>
       </c>
       <c r="J2" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="K2" t="n">
-        <v>651</v>
+        <v>1303</v>
       </c>
       <c r="L2" t="n">
-        <v>39.3</v>
+        <v>39.6</v>
       </c>
       <c r="M2" t="n">
-        <v>70337</v>
+        <v>70988</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -554,34 +554,34 @@
         <v>25030</v>
       </c>
       <c r="D3" t="n">
-        <v>46.9</v>
+        <v>46.2</v>
       </c>
       <c r="E3" t="n">
-        <v>11741</v>
+        <v>11559</v>
       </c>
       <c r="F3" t="n">
-        <v>40</v>
+        <v>33.8</v>
       </c>
       <c r="G3" t="n">
-        <v>10012</v>
+        <v>8465</v>
       </c>
       <c r="H3" t="n">
-        <v>13.1</v>
+        <v>8</v>
       </c>
       <c r="I3" t="n">
-        <v>3277</v>
+        <v>2002</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>3004</v>
       </c>
       <c r="L3" t="n">
-        <v>53.1</v>
+        <v>53.8</v>
       </c>
       <c r="M3" t="n">
-        <v>13289</v>
+        <v>13471</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -609,12 +609,8 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
@@ -643,12 +639,8 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
@@ -784,16 +776,16 @@
         <v>30253</v>
       </c>
       <c r="H8" t="n">
-        <v>5.3</v>
+        <v>2.6</v>
       </c>
       <c r="I8" t="n">
-        <v>4973</v>
+        <v>2487</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>2.6</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>2487</v>
       </c>
       <c r="L8" t="n">
         <v>37.4</v>
@@ -884,16 +876,16 @@
         <v>14809</v>
       </c>
       <c r="H10" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="I10" t="n">
-        <v>793</v>
+        <v>529</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>264</v>
       </c>
       <c r="L10" t="n">
         <v>38.8</v>
@@ -1022,10 +1014,10 @@
         <v>115318</v>
       </c>
       <c r="D13" t="n">
-        <v>58.8</v>
+        <v>58.3</v>
       </c>
       <c r="E13" t="n">
-        <v>67770</v>
+        <v>67223</v>
       </c>
       <c r="F13" t="n">
         <v>37</v>
@@ -1040,16 +1032,16 @@
         <v>4919</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>547</v>
       </c>
       <c r="L13" t="n">
-        <v>41.2</v>
+        <v>41.7</v>
       </c>
       <c r="M13" t="n">
-        <v>47548</v>
+        <v>48095</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -1184,16 +1176,16 @@
         <v>25703</v>
       </c>
       <c r="H16" t="n">
-        <v>11.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="I16" t="n">
-        <v>4698</v>
+        <v>3869</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>829</v>
       </c>
       <c r="L16" t="n">
         <v>72.40000000000001</v>
@@ -1222,34 +1214,34 @@
         <v>75107</v>
       </c>
       <c r="D17" t="n">
-        <v>64.8</v>
+        <v>64.3</v>
       </c>
       <c r="E17" t="n">
-        <v>48641</v>
+        <v>48283</v>
       </c>
       <c r="F17" t="n">
-        <v>26.2</v>
+        <v>25.7</v>
       </c>
       <c r="G17" t="n">
-        <v>19671</v>
+        <v>19313</v>
       </c>
       <c r="H17" t="n">
-        <v>9</v>
+        <v>7.6</v>
       </c>
       <c r="I17" t="n">
-        <v>6795</v>
+        <v>5722</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>1788</v>
       </c>
       <c r="L17" t="n">
-        <v>35.2</v>
+        <v>35.7</v>
       </c>
       <c r="M17" t="n">
-        <v>26466</v>
+        <v>26824</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
@@ -1272,10 +1264,10 @@
         <v>36288</v>
       </c>
       <c r="D18" t="n">
-        <v>83.5</v>
+        <v>82</v>
       </c>
       <c r="E18" t="n">
-        <v>30284</v>
+        <v>29751</v>
       </c>
       <c r="F18" t="n">
         <v>11.4</v>
@@ -1284,22 +1276,22 @@
         <v>4136</v>
       </c>
       <c r="H18" t="n">
-        <v>5.1</v>
+        <v>2.2</v>
       </c>
       <c r="I18" t="n">
-        <v>1868</v>
+        <v>800</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>4.4</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>1601</v>
       </c>
       <c r="L18" t="n">
-        <v>16.5</v>
+        <v>18</v>
       </c>
       <c r="M18" t="n">
-        <v>6004</v>
+        <v>6537</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
@@ -1322,34 +1314,34 @@
         <v>70492</v>
       </c>
       <c r="D19" t="n">
-        <v>16.3</v>
+        <v>15.7</v>
       </c>
       <c r="E19" t="n">
-        <v>11485</v>
+        <v>11089</v>
       </c>
       <c r="F19" t="n">
-        <v>71.3</v>
+        <v>70.8</v>
       </c>
       <c r="G19" t="n">
-        <v>50295</v>
+        <v>49899</v>
       </c>
       <c r="H19" t="n">
-        <v>12.4</v>
+        <v>9</v>
       </c>
       <c r="I19" t="n">
-        <v>8712</v>
+        <v>6336</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>3168</v>
       </c>
       <c r="L19" t="n">
-        <v>83.7</v>
+        <v>84.3</v>
       </c>
       <c r="M19" t="n">
-        <v>59007</v>
+        <v>59403</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -1372,10 +1364,10 @@
         <v>317907</v>
       </c>
       <c r="D20" t="n">
-        <v>49.2</v>
+        <v>47.5</v>
       </c>
       <c r="E20" t="n">
-        <v>156348</v>
+        <v>151136</v>
       </c>
       <c r="F20" t="n">
         <v>48.1</v>
@@ -1390,16 +1382,16 @@
         <v>8686</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>5212</v>
       </c>
       <c r="L20" t="n">
-        <v>50.8</v>
+        <v>52.5</v>
       </c>
       <c r="M20" t="n">
-        <v>161559</v>
+        <v>166771</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -1422,10 +1414,10 @@
         <v>22612</v>
       </c>
       <c r="D21" t="n">
-        <v>65.8</v>
+        <v>65.2</v>
       </c>
       <c r="E21" t="n">
-        <v>14884</v>
+        <v>14741</v>
       </c>
       <c r="F21" t="n">
         <v>34.2</v>
@@ -1440,16 +1432,16 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>143</v>
       </c>
       <c r="L21" t="n">
-        <v>34.2</v>
+        <v>34.8</v>
       </c>
       <c r="M21" t="n">
-        <v>7728</v>
+        <v>7871</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -1472,34 +1464,34 @@
         <v>43076</v>
       </c>
       <c r="D22" t="n">
-        <v>31.6</v>
+        <v>31.2</v>
       </c>
       <c r="E22" t="n">
-        <v>13618</v>
+        <v>13432</v>
       </c>
       <c r="F22" t="n">
-        <v>55.5</v>
+        <v>55.1</v>
       </c>
       <c r="G22" t="n">
-        <v>23900</v>
+        <v>23715</v>
       </c>
       <c r="H22" t="n">
-        <v>12.9</v>
+        <v>6</v>
       </c>
       <c r="I22" t="n">
-        <v>5558</v>
+        <v>2594</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>7.7</v>
       </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>3335</v>
       </c>
       <c r="L22" t="n">
-        <v>68.40000000000001</v>
+        <v>68.8</v>
       </c>
       <c r="M22" t="n">
-        <v>29458</v>
+        <v>29644</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
@@ -1534,16 +1526,16 @@
         <v>17399</v>
       </c>
       <c r="H23" t="n">
-        <v>5.7</v>
+        <v>3.8</v>
       </c>
       <c r="I23" t="n">
-        <v>1535</v>
+        <v>1023</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>512</v>
       </c>
       <c r="L23" t="n">
         <v>69.8</v>
@@ -1577,12 +1569,8 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
@@ -1612,22 +1600,22 @@
         <v>37496</v>
       </c>
       <c r="F25" t="n">
-        <v>41</v>
+        <v>40.5</v>
       </c>
       <c r="G25" t="n">
-        <v>28351</v>
+        <v>28046</v>
       </c>
       <c r="H25" t="n">
-        <v>4.8</v>
+        <v>3.5</v>
       </c>
       <c r="I25" t="n">
-        <v>3353</v>
+        <v>2439</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>1.8</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>1219</v>
       </c>
       <c r="L25" t="n">
         <v>45.8</v>
@@ -1706,10 +1694,10 @@
         <v>56167</v>
       </c>
       <c r="D27" t="n">
-        <v>13.9</v>
+        <v>13</v>
       </c>
       <c r="E27" t="n">
-        <v>7801</v>
+        <v>7281</v>
       </c>
       <c r="F27" t="n">
         <v>83.3</v>
@@ -1718,22 +1706,22 @@
         <v>46806</v>
       </c>
       <c r="H27" t="n">
-        <v>2.8</v>
+        <v>1.9</v>
       </c>
       <c r="I27" t="n">
-        <v>1560</v>
+        <v>1040</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="K27" t="n">
-        <v>0</v>
+        <v>1040</v>
       </c>
       <c r="L27" t="n">
-        <v>86.09999999999999</v>
+        <v>87</v>
       </c>
       <c r="M27" t="n">
-        <v>48366</v>
+        <v>48886</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
@@ -1768,16 +1756,16 @@
         <v>14321</v>
       </c>
       <c r="H28" t="n">
-        <v>6.6</v>
+        <v>4.5</v>
       </c>
       <c r="I28" t="n">
-        <v>5032</v>
+        <v>3484</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>1548</v>
       </c>
       <c r="L28" t="n">
         <v>25.3</v>
@@ -1806,10 +1794,10 @@
         <v>326014</v>
       </c>
       <c r="D29" t="n">
-        <v>62.3</v>
+        <v>61.7</v>
       </c>
       <c r="E29" t="n">
-        <v>203091</v>
+        <v>201309</v>
       </c>
       <c r="F29" t="n">
         <v>27.3</v>
@@ -1818,22 +1806,22 @@
         <v>89075</v>
       </c>
       <c r="H29" t="n">
-        <v>10.4</v>
+        <v>5.5</v>
       </c>
       <c r="I29" t="n">
-        <v>33848</v>
+        <v>17815</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>17815</v>
       </c>
       <c r="L29" t="n">
-        <v>37.7</v>
+        <v>38.3</v>
       </c>
       <c r="M29" t="n">
-        <v>122923</v>
+        <v>124705</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
@@ -1856,10 +1844,10 @@
         <v>79290</v>
       </c>
       <c r="D30" t="n">
-        <v>63.6</v>
+        <v>63</v>
       </c>
       <c r="E30" t="n">
-        <v>50413</v>
+        <v>49923</v>
       </c>
       <c r="F30" t="n">
         <v>28.7</v>
@@ -1874,16 +1862,16 @@
         <v>6118</v>
       </c>
       <c r="J30" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K30" t="n">
-        <v>0</v>
+        <v>489</v>
       </c>
       <c r="L30" t="n">
-        <v>36.4</v>
+        <v>37</v>
       </c>
       <c r="M30" t="n">
-        <v>28877</v>
+        <v>29367</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
@@ -1906,10 +1894,10 @@
         <v>86213</v>
       </c>
       <c r="D31" t="n">
-        <v>58.2</v>
+        <v>57.7</v>
       </c>
       <c r="E31" t="n">
-        <v>50212</v>
+        <v>49738</v>
       </c>
       <c r="F31" t="n">
         <v>40.7</v>
@@ -1924,16 +1912,16 @@
         <v>947</v>
       </c>
       <c r="J31" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K31" t="n">
-        <v>0</v>
+        <v>474</v>
       </c>
       <c r="L31" t="n">
-        <v>41.8</v>
+        <v>42.3</v>
       </c>
       <c r="M31" t="n">
-        <v>36001</v>
+        <v>36475</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -2011,12 +1999,8 @@
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" t="n">
-        <v>0</v>
-      </c>
-      <c r="K33" t="n">
-        <v>0</v>
-      </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr">
@@ -2052,16 +2036,16 @@
         <v>38681</v>
       </c>
       <c r="H34" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="I34" t="n">
-        <v>3339</v>
+        <v>2505</v>
       </c>
       <c r="J34" t="n">
-        <v>0.6</v>
+        <v>1.4</v>
       </c>
       <c r="K34" t="n">
-        <v>557</v>
+        <v>1391</v>
       </c>
       <c r="L34" t="n">
         <v>42.3</v>
@@ -2090,10 +2074,10 @@
         <v>79093</v>
       </c>
       <c r="D35" t="n">
-        <v>61.8</v>
+        <v>61.3</v>
       </c>
       <c r="E35" t="n">
-        <v>48902</v>
+        <v>48476</v>
       </c>
       <c r="F35" t="n">
         <v>34.9</v>
@@ -2102,22 +2086,22 @@
         <v>27640</v>
       </c>
       <c r="H35" t="n">
-        <v>3.2</v>
+        <v>1.6</v>
       </c>
       <c r="I35" t="n">
-        <v>2551</v>
+        <v>1276</v>
       </c>
       <c r="J35" t="n">
-        <v>0</v>
+        <v>2.2</v>
       </c>
       <c r="K35" t="n">
-        <v>0</v>
+        <v>1701</v>
       </c>
       <c r="L35" t="n">
-        <v>38.2</v>
+        <v>38.7</v>
       </c>
       <c r="M35" t="n">
-        <v>30191</v>
+        <v>30617</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
@@ -2140,10 +2124,10 @@
         <v>59428</v>
       </c>
       <c r="D36" t="n">
-        <v>71.59999999999999</v>
+        <v>71</v>
       </c>
       <c r="E36" t="n">
-        <v>42522</v>
+        <v>42180</v>
       </c>
       <c r="F36" t="n">
         <v>25.6</v>
@@ -2152,22 +2136,22 @@
         <v>15199</v>
       </c>
       <c r="H36" t="n">
-        <v>2.9</v>
+        <v>2.6</v>
       </c>
       <c r="I36" t="n">
-        <v>1708</v>
+        <v>1537</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>512</v>
       </c>
       <c r="L36" t="n">
-        <v>28.4</v>
+        <v>29</v>
       </c>
       <c r="M36" t="n">
-        <v>16906</v>
+        <v>17248</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
@@ -2229,12 +2213,8 @@
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" t="n">
-        <v>0</v>
-      </c>
-      <c r="K38" t="n">
-        <v>0</v>
-      </c>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
@@ -2270,16 +2250,16 @@
         <v>88265</v>
       </c>
       <c r="H39" t="n">
-        <v>3</v>
+        <v>1.7</v>
       </c>
       <c r="I39" t="n">
-        <v>4045</v>
+        <v>2207</v>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="K39" t="n">
-        <v>0</v>
+        <v>1839</v>
       </c>
       <c r="L39" t="n">
         <v>69.3</v>
@@ -2313,12 +2293,8 @@
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" t="n">
-        <v>0</v>
-      </c>
-      <c r="K40" t="n">
-        <v>0</v>
-      </c>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr">
@@ -2348,22 +2324,22 @@
         <v>819</v>
       </c>
       <c r="F41" t="n">
-        <v>88.59999999999999</v>
+        <v>88</v>
       </c>
       <c r="G41" t="n">
-        <v>24247</v>
+        <v>24083</v>
       </c>
       <c r="H41" t="n">
-        <v>8.4</v>
+        <v>4.8</v>
       </c>
       <c r="I41" t="n">
-        <v>2294</v>
+        <v>1311</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>4.2</v>
       </c>
       <c r="K41" t="n">
-        <v>0</v>
+        <v>1147</v>
       </c>
       <c r="L41" t="n">
         <v>97</v>
@@ -2392,10 +2368,10 @@
         <v>172940</v>
       </c>
       <c r="D42" t="n">
-        <v>41.1</v>
+        <v>40.7</v>
       </c>
       <c r="E42" t="n">
-        <v>71162</v>
+        <v>70334</v>
       </c>
       <c r="F42" t="n">
         <v>41.6</v>
@@ -2404,22 +2380,22 @@
         <v>71989</v>
       </c>
       <c r="H42" t="n">
-        <v>17.2</v>
+        <v>10</v>
       </c>
       <c r="I42" t="n">
-        <v>29789</v>
+        <v>17377</v>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
+        <v>7.7</v>
       </c>
       <c r="K42" t="n">
-        <v>0</v>
+        <v>13239</v>
       </c>
       <c r="L42" t="n">
-        <v>58.9</v>
+        <v>59.3</v>
       </c>
       <c r="M42" t="n">
-        <v>101778</v>
+        <v>102606</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
@@ -2447,12 +2423,8 @@
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr"/>
-      <c r="J43" t="n">
-        <v>0</v>
-      </c>
-      <c r="K43" t="n">
-        <v>0</v>
-      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
@@ -2481,12 +2453,8 @@
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr"/>
-      <c r="J44" t="n">
-        <v>0</v>
-      </c>
-      <c r="K44" t="n">
-        <v>0</v>
-      </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr">
@@ -2515,12 +2483,8 @@
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr"/>
-      <c r="J45" t="n">
-        <v>0</v>
-      </c>
-      <c r="K45" t="n">
-        <v>0</v>
-      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr">
@@ -2544,10 +2508,10 @@
         <v>6160</v>
       </c>
       <c r="D46" t="n">
-        <v>73.2</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="E46" t="n">
-        <v>4509</v>
+        <v>4460</v>
       </c>
       <c r="F46" t="n">
         <v>20.4</v>
@@ -2556,22 +2520,22 @@
         <v>1257</v>
       </c>
       <c r="H46" t="n">
-        <v>6.4</v>
+        <v>0</v>
       </c>
       <c r="I46" t="n">
-        <v>394</v>
+        <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="K46" t="n">
-        <v>0</v>
+        <v>444</v>
       </c>
       <c r="L46" t="n">
-        <v>26.8</v>
+        <v>27.6</v>
       </c>
       <c r="M46" t="n">
-        <v>1651</v>
+        <v>1700</v>
       </c>
       <c r="N46" t="inlineStr">
         <is>
@@ -2594,34 +2558,34 @@
         <v>29929</v>
       </c>
       <c r="D47" t="n">
-        <v>65.09999999999999</v>
+        <v>63.4</v>
       </c>
       <c r="E47" t="n">
-        <v>19486</v>
+        <v>18976</v>
       </c>
       <c r="F47" t="n">
-        <v>24.3</v>
+        <v>23.8</v>
       </c>
       <c r="G47" t="n">
-        <v>7259</v>
+        <v>7132</v>
       </c>
       <c r="H47" t="n">
-        <v>10.6</v>
+        <v>9.4</v>
       </c>
       <c r="I47" t="n">
-        <v>3184</v>
+        <v>2802</v>
       </c>
       <c r="J47" t="n">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="K47" t="n">
-        <v>0</v>
+        <v>1019</v>
       </c>
       <c r="L47" t="n">
-        <v>34.9</v>
+        <v>36.6</v>
       </c>
       <c r="M47" t="n">
-        <v>10443</v>
+        <v>10953</v>
       </c>
       <c r="N47" t="inlineStr">
         <is>
@@ -2644,34 +2608,34 @@
         <v>102440</v>
       </c>
       <c r="D48" t="n">
-        <v>40.6</v>
+        <v>39.1</v>
       </c>
       <c r="E48" t="n">
-        <v>41600</v>
+        <v>40040</v>
       </c>
       <c r="F48" t="n">
-        <v>54.3</v>
+        <v>53.8</v>
       </c>
       <c r="G48" t="n">
-        <v>55640</v>
+        <v>55120</v>
       </c>
       <c r="H48" t="n">
-        <v>5.1</v>
+        <v>4.1</v>
       </c>
       <c r="I48" t="n">
-        <v>5200</v>
+        <v>4160</v>
       </c>
       <c r="J48" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K48" t="n">
-        <v>0</v>
+        <v>3120</v>
       </c>
       <c r="L48" t="n">
-        <v>59.4</v>
+        <v>60.9</v>
       </c>
       <c r="M48" t="n">
-        <v>60840</v>
+        <v>62400</v>
       </c>
       <c r="N48" t="inlineStr">
         <is>
@@ -2694,10 +2658,10 @@
         <v>46949</v>
       </c>
       <c r="D49" t="n">
-        <v>56.6</v>
+        <v>55.2</v>
       </c>
       <c r="E49" t="n">
-        <v>26588</v>
+        <v>25915</v>
       </c>
       <c r="F49" t="n">
         <v>36.2</v>
@@ -2706,22 +2670,22 @@
         <v>16996</v>
       </c>
       <c r="H49" t="n">
-        <v>6.8</v>
+        <v>5</v>
       </c>
       <c r="I49" t="n">
-        <v>3197</v>
+        <v>2356</v>
       </c>
       <c r="J49" t="n">
-        <v>0.4</v>
+        <v>3.6</v>
       </c>
       <c r="K49" t="n">
-        <v>168</v>
+        <v>1683</v>
       </c>
       <c r="L49" t="n">
-        <v>43.4</v>
+        <v>44.8</v>
       </c>
       <c r="M49" t="n">
-        <v>20361</v>
+        <v>21034</v>
       </c>
       <c r="N49" t="inlineStr">
         <is>
@@ -2744,10 +2708,10 @@
         <v>21140</v>
       </c>
       <c r="D50" t="n">
-        <v>68.3</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="E50" t="n">
-        <v>14442</v>
+        <v>14283</v>
       </c>
       <c r="F50" t="n">
         <v>25.3</v>
@@ -2756,22 +2720,22 @@
         <v>5359</v>
       </c>
       <c r="H50" t="n">
-        <v>6.3</v>
+        <v>2.6</v>
       </c>
       <c r="I50" t="n">
-        <v>1340</v>
+        <v>545</v>
       </c>
       <c r="J50" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="K50" t="n">
-        <v>0</v>
+        <v>954</v>
       </c>
       <c r="L50" t="n">
-        <v>31.7</v>
+        <v>32.4</v>
       </c>
       <c r="M50" t="n">
-        <v>6698</v>
+        <v>6857</v>
       </c>
       <c r="N50" t="inlineStr">
         <is>
@@ -2794,34 +2758,34 @@
         <v>31281</v>
       </c>
       <c r="D51" t="n">
-        <v>49.8</v>
+        <v>47.8</v>
       </c>
       <c r="E51" t="n">
-        <v>15587</v>
+        <v>14947</v>
       </c>
       <c r="F51" t="n">
-        <v>44.7</v>
+        <v>44.4</v>
       </c>
       <c r="G51" t="n">
-        <v>13986</v>
+        <v>13879</v>
       </c>
       <c r="H51" t="n">
-        <v>5.1</v>
+        <v>4.1</v>
       </c>
       <c r="I51" t="n">
-        <v>1601</v>
+        <v>1281</v>
       </c>
       <c r="J51" t="n">
-        <v>0.3</v>
+        <v>3.8</v>
       </c>
       <c r="K51" t="n">
-        <v>107</v>
+        <v>1174</v>
       </c>
       <c r="L51" t="n">
-        <v>50.2</v>
+        <v>52.2</v>
       </c>
       <c r="M51" t="n">
-        <v>15694</v>
+        <v>16334</v>
       </c>
       <c r="N51" t="inlineStr">
         <is>
@@ -2844,10 +2808,10 @@
         <v>48858</v>
       </c>
       <c r="D52" t="n">
-        <v>67.09999999999999</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="E52" t="n">
-        <v>32794</v>
+        <v>32461</v>
       </c>
       <c r="F52" t="n">
         <v>29.7</v>
@@ -2856,22 +2820,22 @@
         <v>14513</v>
       </c>
       <c r="H52" t="n">
-        <v>3.2</v>
+        <v>2.3</v>
       </c>
       <c r="I52" t="n">
-        <v>1551</v>
+        <v>1108</v>
       </c>
       <c r="J52" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="K52" t="n">
-        <v>0</v>
+        <v>776</v>
       </c>
       <c r="L52" t="n">
-        <v>32.9</v>
+        <v>33.6</v>
       </c>
       <c r="M52" t="n">
-        <v>16064</v>
+        <v>16397</v>
       </c>
       <c r="N52" t="inlineStr">
         <is>
@@ -2894,34 +2858,34 @@
         <v>31931</v>
       </c>
       <c r="D53" t="n">
-        <v>68.40000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="E53" t="n">
-        <v>21832</v>
+        <v>21640</v>
       </c>
       <c r="F53" t="n">
-        <v>22.6</v>
+        <v>22.3</v>
       </c>
       <c r="G53" t="n">
-        <v>7213</v>
+        <v>7117</v>
       </c>
       <c r="H53" t="n">
-        <v>9</v>
+        <v>6.6</v>
       </c>
       <c r="I53" t="n">
-        <v>2885</v>
+        <v>2116</v>
       </c>
       <c r="J53" t="n">
-        <v>0</v>
+        <v>3.3</v>
       </c>
       <c r="K53" t="n">
-        <v>0</v>
+        <v>1058</v>
       </c>
       <c r="L53" t="n">
-        <v>31.6</v>
+        <v>32.2</v>
       </c>
       <c r="M53" t="n">
-        <v>10099</v>
+        <v>10291</v>
       </c>
       <c r="N53" t="inlineStr">
         <is>
@@ -2944,10 +2908,10 @@
         <v>160918</v>
       </c>
       <c r="D54" t="n">
-        <v>64.7</v>
+        <v>62.4</v>
       </c>
       <c r="E54" t="n">
-        <v>104192</v>
+        <v>100333</v>
       </c>
       <c r="F54" t="n">
         <v>25.7</v>
@@ -2956,22 +2920,22 @@
         <v>41291</v>
       </c>
       <c r="H54" t="n">
-        <v>9.6</v>
+        <v>6</v>
       </c>
       <c r="I54" t="n">
-        <v>15436</v>
+        <v>9647</v>
       </c>
       <c r="J54" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K54" t="n">
-        <v>0</v>
+        <v>9647</v>
       </c>
       <c r="L54" t="n">
-        <v>35.3</v>
+        <v>37.6</v>
       </c>
       <c r="M54" t="n">
-        <v>56726</v>
+        <v>60585</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
@@ -3000,19 +2964,19 @@
         <v>0</v>
       </c>
       <c r="F55" t="n">
-        <v>43</v>
+        <v>42.2</v>
       </c>
       <c r="G55" t="n">
         <v>0</v>
       </c>
       <c r="H55" t="n">
-        <v>9.1</v>
+        <v>6.5</v>
       </c>
       <c r="I55" t="n">
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="K55" t="n">
         <v>0</v>
@@ -3044,10 +3008,10 @@
         <v>56819</v>
       </c>
       <c r="D56" t="n">
-        <v>63.4</v>
+        <v>62.4</v>
       </c>
       <c r="E56" t="n">
-        <v>36014</v>
+        <v>35440</v>
       </c>
       <c r="F56" t="n">
         <v>28.3</v>
@@ -3056,22 +3020,22 @@
         <v>16070</v>
       </c>
       <c r="H56" t="n">
-        <v>8.300000000000001</v>
+        <v>2.5</v>
       </c>
       <c r="I56" t="n">
-        <v>4735</v>
+        <v>1435</v>
       </c>
       <c r="J56" t="n">
-        <v>0</v>
+        <v>6.8</v>
       </c>
       <c r="K56" t="n">
-        <v>0</v>
+        <v>3874</v>
       </c>
       <c r="L56" t="n">
-        <v>36.6</v>
+        <v>37.6</v>
       </c>
       <c r="M56" t="n">
-        <v>20805</v>
+        <v>21379</v>
       </c>
       <c r="N56" t="inlineStr">
         <is>
@@ -3094,34 +3058,34 @@
         <v>11326</v>
       </c>
       <c r="D57" t="n">
-        <v>72.59999999999999</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="E57" t="n">
-        <v>8218</v>
+        <v>8165</v>
       </c>
       <c r="F57" t="n">
-        <v>20.5</v>
+        <v>19.5</v>
       </c>
       <c r="G57" t="n">
-        <v>2318</v>
+        <v>2213</v>
       </c>
       <c r="H57" t="n">
-        <v>6.5</v>
+        <v>4.7</v>
       </c>
       <c r="I57" t="n">
-        <v>738</v>
+        <v>527</v>
       </c>
       <c r="J57" t="n">
-        <v>0.5</v>
+        <v>3.7</v>
       </c>
       <c r="K57" t="n">
-        <v>53</v>
+        <v>421</v>
       </c>
       <c r="L57" t="n">
-        <v>27.4</v>
+        <v>27.9</v>
       </c>
       <c r="M57" t="n">
-        <v>3108</v>
+        <v>3161</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
@@ -3144,34 +3108,34 @@
         <v>55986</v>
       </c>
       <c r="D58" t="n">
-        <v>68.59999999999999</v>
+        <v>68.3</v>
       </c>
       <c r="E58" t="n">
-        <v>38402</v>
+        <v>38244</v>
       </c>
       <c r="F58" t="n">
-        <v>24.9</v>
+        <v>24.5</v>
       </c>
       <c r="G58" t="n">
-        <v>13957</v>
+        <v>13721</v>
       </c>
       <c r="H58" t="n">
-        <v>6.3</v>
+        <v>3</v>
       </c>
       <c r="I58" t="n">
-        <v>3548</v>
+        <v>1656</v>
       </c>
       <c r="J58" t="n">
-        <v>0.1</v>
+        <v>4.2</v>
       </c>
       <c r="K58" t="n">
-        <v>79</v>
+        <v>2366</v>
       </c>
       <c r="L58" t="n">
-        <v>31.4</v>
+        <v>31.7</v>
       </c>
       <c r="M58" t="n">
-        <v>17584</v>
+        <v>17742</v>
       </c>
       <c r="N58" t="inlineStr">
         <is>
@@ -3194,34 +3158,34 @@
         <v>29679</v>
       </c>
       <c r="D59" t="n">
-        <v>63.8</v>
+        <v>62.7</v>
       </c>
       <c r="E59" t="n">
-        <v>18921</v>
+        <v>18616</v>
       </c>
       <c r="F59" t="n">
-        <v>27.2</v>
+        <v>27</v>
       </c>
       <c r="G59" t="n">
-        <v>8087</v>
+        <v>8011</v>
       </c>
       <c r="H59" t="n">
-        <v>9</v>
+        <v>6.2</v>
       </c>
       <c r="I59" t="n">
-        <v>2670</v>
+        <v>1831</v>
       </c>
       <c r="J59" t="n">
-        <v>0</v>
+        <v>4.1</v>
       </c>
       <c r="K59" t="n">
-        <v>0</v>
+        <v>1221</v>
       </c>
       <c r="L59" t="n">
-        <v>36.2</v>
+        <v>37.3</v>
       </c>
       <c r="M59" t="n">
-        <v>10758</v>
+        <v>11063</v>
       </c>
       <c r="N59" t="inlineStr">
         <is>
@@ -3244,10 +3208,10 @@
         <v>246091</v>
       </c>
       <c r="D60" t="n">
-        <v>56.4</v>
+        <v>55.3</v>
       </c>
       <c r="E60" t="n">
-        <v>138856</v>
+        <v>136106</v>
       </c>
       <c r="F60" t="n">
         <v>38.5</v>
@@ -3256,22 +3220,22 @@
         <v>94862</v>
       </c>
       <c r="H60" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="I60" t="n">
-        <v>12373</v>
+        <v>10998</v>
       </c>
       <c r="J60" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="K60" t="n">
-        <v>0</v>
+        <v>4124</v>
       </c>
       <c r="L60" t="n">
-        <v>43.6</v>
+        <v>44.7</v>
       </c>
       <c r="M60" t="n">
-        <v>107235</v>
+        <v>109985</v>
       </c>
       <c r="N60" t="inlineStr">
         <is>
@@ -3294,34 +3258,34 @@
         <v>49364</v>
       </c>
       <c r="D61" t="n">
-        <v>68.5</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="E61" t="n">
-        <v>33817</v>
+        <v>33363</v>
       </c>
       <c r="F61" t="n">
-        <v>26</v>
+        <v>25.5</v>
       </c>
       <c r="G61" t="n">
-        <v>12823</v>
+        <v>12596</v>
       </c>
       <c r="H61" t="n">
-        <v>5.5</v>
+        <v>2.8</v>
       </c>
       <c r="I61" t="n">
-        <v>2724</v>
+        <v>1362</v>
       </c>
       <c r="J61" t="n">
-        <v>0</v>
+        <v>4.1</v>
       </c>
       <c r="K61" t="n">
-        <v>0</v>
+        <v>2043</v>
       </c>
       <c r="L61" t="n">
-        <v>31.5</v>
+        <v>32.4</v>
       </c>
       <c r="M61" t="n">
-        <v>15547</v>
+        <v>16001</v>
       </c>
       <c r="N61" t="inlineStr">
         <is>
@@ -3356,16 +3320,16 @@
         <v>9829</v>
       </c>
       <c r="H62" t="n">
-        <v>7.5</v>
+        <v>2.4</v>
       </c>
       <c r="I62" t="n">
-        <v>2837</v>
+        <v>912</v>
       </c>
       <c r="J62" t="n">
-        <v>0</v>
+        <v>5.1</v>
       </c>
       <c r="K62" t="n">
-        <v>0</v>
+        <v>1925</v>
       </c>
       <c r="L62" t="n">
         <v>33.4</v>
@@ -3394,10 +3358,10 @@
         <v>123497</v>
       </c>
       <c r="D63" t="n">
-        <v>54.5</v>
+        <v>54.2</v>
       </c>
       <c r="E63" t="n">
-        <v>67362</v>
+        <v>66961</v>
       </c>
       <c r="F63" t="n">
         <v>43.8</v>
@@ -3406,22 +3370,22 @@
         <v>54130</v>
       </c>
       <c r="H63" t="n">
-        <v>1.6</v>
+        <v>0.6</v>
       </c>
       <c r="I63" t="n">
-        <v>2005</v>
+        <v>802</v>
       </c>
       <c r="J63" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="K63" t="n">
-        <v>0</v>
+        <v>1604</v>
       </c>
       <c r="L63" t="n">
-        <v>45.5</v>
+        <v>45.8</v>
       </c>
       <c r="M63" t="n">
-        <v>56135</v>
+        <v>56536</v>
       </c>
       <c r="N63" t="inlineStr">
         <is>
@@ -3444,10 +3408,10 @@
         <v>227654</v>
       </c>
       <c r="D64" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="E64" t="n">
-        <v>57384</v>
+        <v>53621</v>
       </c>
       <c r="F64" t="n">
         <v>62.4</v>
@@ -3456,22 +3420,22 @@
         <v>142049</v>
       </c>
       <c r="H64" t="n">
-        <v>12</v>
+        <v>10.7</v>
       </c>
       <c r="I64" t="n">
-        <v>27281</v>
+        <v>24459</v>
       </c>
       <c r="J64" t="n">
-        <v>0.4</v>
+        <v>3.3</v>
       </c>
       <c r="K64" t="n">
-        <v>941</v>
+        <v>7526</v>
       </c>
       <c r="L64" t="n">
-        <v>74.8</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="M64" t="n">
-        <v>170270</v>
+        <v>174033</v>
       </c>
       <c r="N64" t="inlineStr">
         <is>
@@ -3617,12 +3581,8 @@
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr"/>
-      <c r="J68" t="n">
-        <v>0</v>
-      </c>
-      <c r="K68" t="n">
-        <v>0</v>
-      </c>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr"/>
       <c r="N68" t="inlineStr">
@@ -3646,10 +3606,10 @@
         <v>167182</v>
       </c>
       <c r="D69" t="n">
-        <v>7.2</v>
+        <v>6.4</v>
       </c>
       <c r="E69" t="n">
-        <v>12094</v>
+        <v>10671</v>
       </c>
       <c r="F69" t="n">
         <v>60.4</v>
@@ -3658,22 +3618,22 @@
         <v>101021</v>
       </c>
       <c r="H69" t="n">
-        <v>32.3</v>
+        <v>27.7</v>
       </c>
       <c r="I69" t="n">
-        <v>54067</v>
+        <v>46242</v>
       </c>
       <c r="J69" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="K69" t="n">
-        <v>0</v>
+        <v>9248</v>
       </c>
       <c r="L69" t="n">
-        <v>92.8</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="M69" t="n">
-        <v>155088</v>
+        <v>156511</v>
       </c>
       <c r="N69" t="inlineStr">
         <is>
@@ -3696,34 +3656,34 @@
         <v>114149</v>
       </c>
       <c r="D70" t="n">
-        <v>38.1</v>
+        <v>36.5</v>
       </c>
       <c r="E70" t="n">
-        <v>43515</v>
+        <v>41623</v>
       </c>
       <c r="F70" t="n">
-        <v>53</v>
+        <v>52.5</v>
       </c>
       <c r="G70" t="n">
-        <v>60543</v>
+        <v>59912</v>
       </c>
       <c r="H70" t="n">
-        <v>8.800000000000001</v>
+        <v>1.7</v>
       </c>
       <c r="I70" t="n">
-        <v>10091</v>
+        <v>1892</v>
       </c>
       <c r="J70" t="n">
-        <v>0</v>
+        <v>9.4</v>
       </c>
       <c r="K70" t="n">
-        <v>0</v>
+        <v>10721</v>
       </c>
       <c r="L70" t="n">
-        <v>61.9</v>
+        <v>63.5</v>
       </c>
       <c r="M70" t="n">
-        <v>70634</v>
+        <v>72526</v>
       </c>
       <c r="N70" t="inlineStr">
         <is>
@@ -3746,10 +3706,10 @@
         <v>90174</v>
       </c>
       <c r="D71" t="n">
-        <v>42</v>
+        <v>41.4</v>
       </c>
       <c r="E71" t="n">
-        <v>37911</v>
+        <v>37369</v>
       </c>
       <c r="F71" t="n">
         <v>52.9</v>
@@ -3758,22 +3718,22 @@
         <v>47660</v>
       </c>
       <c r="H71" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I71" t="n">
+        <v>542</v>
+      </c>
+      <c r="J71" t="n">
         <v>5.1</v>
       </c>
-      <c r="I71" t="n">
+      <c r="K71" t="n">
         <v>4603</v>
       </c>
-      <c r="J71" t="n">
-        <v>0</v>
-      </c>
-      <c r="K71" t="n">
-        <v>0</v>
-      </c>
       <c r="L71" t="n">
-        <v>58</v>
+        <v>58.6</v>
       </c>
       <c r="M71" t="n">
-        <v>52263</v>
+        <v>52805</v>
       </c>
       <c r="N71" t="inlineStr">
         <is>
@@ -3796,10 +3756,10 @@
         <v>68073</v>
       </c>
       <c r="D72" t="n">
-        <v>43.4</v>
+        <v>43</v>
       </c>
       <c r="E72" t="n">
-        <v>29526</v>
+        <v>29252</v>
       </c>
       <c r="F72" t="n">
         <v>55</v>
@@ -3814,16 +3774,16 @@
         <v>820</v>
       </c>
       <c r="J72" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="K72" t="n">
-        <v>273</v>
+        <v>547</v>
       </c>
       <c r="L72" t="n">
-        <v>56.6</v>
+        <v>57</v>
       </c>
       <c r="M72" t="n">
-        <v>38547</v>
+        <v>38821</v>
       </c>
       <c r="N72" t="inlineStr">
         <is>
@@ -3852,22 +3812,22 @@
         <v>17198</v>
       </c>
       <c r="F73" t="n">
-        <v>55.3</v>
+        <v>54.8</v>
       </c>
       <c r="G73" t="n">
-        <v>22521</v>
+        <v>22317</v>
       </c>
       <c r="H73" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="I73" t="n">
-        <v>1024</v>
+        <v>819</v>
       </c>
       <c r="J73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K73" t="n">
-        <v>0</v>
+        <v>409</v>
       </c>
       <c r="L73" t="n">
         <v>57.8</v>
@@ -3896,34 +3856,34 @@
         <v>30087</v>
       </c>
       <c r="D74" t="n">
-        <v>24.7</v>
+        <v>24.4</v>
       </c>
       <c r="E74" t="n">
-        <v>7423</v>
+        <v>7344</v>
       </c>
       <c r="F74" t="n">
-        <v>72.2</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="G74" t="n">
-        <v>21716</v>
+        <v>21637</v>
       </c>
       <c r="H74" t="n">
-        <v>3.1</v>
+        <v>2.6</v>
       </c>
       <c r="I74" t="n">
-        <v>948</v>
+        <v>790</v>
       </c>
       <c r="J74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K74" t="n">
-        <v>0</v>
+        <v>316</v>
       </c>
       <c r="L74" t="n">
-        <v>75.3</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="M74" t="n">
-        <v>22664</v>
+        <v>22743</v>
       </c>
       <c r="N74" t="inlineStr">
         <is>
@@ -3958,16 +3918,16 @@
         <v>15865</v>
       </c>
       <c r="H75" t="n">
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="I75" t="n">
-        <v>3690</v>
+        <v>3505</v>
       </c>
       <c r="J75" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K75" t="n">
-        <v>0</v>
+        <v>184</v>
       </c>
       <c r="L75" t="n">
         <v>55.8</v>
@@ -4001,12 +3961,8 @@
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr"/>
       <c r="I76" t="inlineStr"/>
-      <c r="J76" t="n">
-        <v>0</v>
-      </c>
-      <c r="K76" t="n">
-        <v>0</v>
-      </c>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr"/>
       <c r="M76" t="inlineStr"/>
       <c r="N76" t="inlineStr">
@@ -4030,10 +3986,10 @@
         <v>35536</v>
       </c>
       <c r="D77" t="n">
-        <v>39.2</v>
+        <v>38.8</v>
       </c>
       <c r="E77" t="n">
-        <v>13940</v>
+        <v>13779</v>
       </c>
       <c r="F77" t="n">
         <v>50.6</v>
@@ -4042,22 +3998,22 @@
         <v>17969</v>
       </c>
       <c r="H77" t="n">
-        <v>10.2</v>
+        <v>8.6</v>
       </c>
       <c r="I77" t="n">
-        <v>3626</v>
+        <v>3062</v>
       </c>
       <c r="J77" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K77" t="n">
-        <v>0</v>
+        <v>725</v>
       </c>
       <c r="L77" t="n">
-        <v>60.8</v>
+        <v>61.2</v>
       </c>
       <c r="M77" t="n">
-        <v>21596</v>
+        <v>21757</v>
       </c>
       <c r="N77" t="inlineStr">
         <is>
@@ -4085,12 +4041,8 @@
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr"/>
-      <c r="J78" t="n">
-        <v>0</v>
-      </c>
-      <c r="K78" t="n">
-        <v>0</v>
-      </c>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr"/>
       <c r="M78" t="inlineStr"/>
       <c r="N78" t="inlineStr">
@@ -4114,10 +4066,10 @@
         <v>62595</v>
       </c>
       <c r="D79" t="n">
-        <v>61.4</v>
+        <v>60.2</v>
       </c>
       <c r="E79" t="n">
-        <v>38444</v>
+        <v>37705</v>
       </c>
       <c r="F79" t="n">
         <v>27.6</v>
@@ -4126,22 +4078,22 @@
         <v>17251</v>
       </c>
       <c r="H79" t="n">
-        <v>11</v>
+        <v>9.4</v>
       </c>
       <c r="I79" t="n">
-        <v>6900</v>
+        <v>5914</v>
       </c>
       <c r="J79" t="n">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="K79" t="n">
-        <v>0</v>
+        <v>1725</v>
       </c>
       <c r="L79" t="n">
-        <v>38.6</v>
+        <v>39.8</v>
       </c>
       <c r="M79" t="n">
-        <v>24151</v>
+        <v>24890</v>
       </c>
       <c r="N79" t="inlineStr">
         <is>
@@ -4170,10 +4122,10 @@
         <v>30395</v>
       </c>
       <c r="F80" t="n">
-        <v>42.3</v>
+        <v>41.1</v>
       </c>
       <c r="G80" t="n">
-        <v>23768</v>
+        <v>23082</v>
       </c>
       <c r="H80" t="n">
         <v>3.7</v>
@@ -4182,10 +4134,10 @@
         <v>2057</v>
       </c>
       <c r="J80" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="K80" t="n">
-        <v>0</v>
+        <v>686</v>
       </c>
       <c r="L80" t="n">
         <v>45.9</v>
@@ -4219,12 +4171,8 @@
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr"/>
-      <c r="J81" t="n">
-        <v>0</v>
-      </c>
-      <c r="K81" t="n">
-        <v>0</v>
-      </c>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr"/>
       <c r="M81" t="inlineStr"/>
       <c r="N81" t="inlineStr">
@@ -4248,10 +4196,10 @@
         <v>40699</v>
       </c>
       <c r="D82" t="n">
-        <v>58.7</v>
+        <v>57.4</v>
       </c>
       <c r="E82" t="n">
-        <v>23900</v>
+        <v>23366</v>
       </c>
       <c r="F82" t="n">
         <v>30.4</v>
@@ -4260,22 +4208,22 @@
         <v>12370</v>
       </c>
       <c r="H82" t="n">
-        <v>10.9</v>
+        <v>10.7</v>
       </c>
       <c r="I82" t="n">
-        <v>4429</v>
+        <v>4352</v>
       </c>
       <c r="J82" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="K82" t="n">
-        <v>0</v>
+        <v>611</v>
       </c>
       <c r="L82" t="n">
-        <v>41.3</v>
+        <v>42.6</v>
       </c>
       <c r="M82" t="n">
-        <v>16799</v>
+        <v>17333</v>
       </c>
       <c r="N82" t="inlineStr">
         <is>
@@ -4298,10 +4246,10 @@
         <v>36859</v>
       </c>
       <c r="D83" t="n">
-        <v>47</v>
+        <v>46.7</v>
       </c>
       <c r="E83" t="n">
-        <v>17330</v>
+        <v>17201</v>
       </c>
       <c r="F83" t="n">
         <v>29.1</v>
@@ -4310,22 +4258,22 @@
         <v>10734</v>
       </c>
       <c r="H83" t="n">
-        <v>23.9</v>
+        <v>17.2</v>
       </c>
       <c r="I83" t="n">
-        <v>8794</v>
+        <v>6337</v>
       </c>
       <c r="J83" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K83" t="n">
-        <v>0</v>
+        <v>2587</v>
       </c>
       <c r="L83" t="n">
-        <v>53</v>
+        <v>53.3</v>
       </c>
       <c r="M83" t="n">
-        <v>19529</v>
+        <v>19658</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
@@ -4433,12 +4381,8 @@
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr"/>
-      <c r="J86" t="n">
-        <v>0</v>
-      </c>
-      <c r="K86" t="n">
-        <v>0</v>
-      </c>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr"/>
       <c r="M86" t="inlineStr"/>
       <c r="N86" t="inlineStr">
@@ -4496,10 +4440,10 @@
         <v>79724</v>
       </c>
       <c r="D88" t="n">
-        <v>64.2</v>
+        <v>63.9</v>
       </c>
       <c r="E88" t="n">
-        <v>51189</v>
+        <v>50971</v>
       </c>
       <c r="F88" t="n">
         <v>32.2</v>
@@ -4508,22 +4452,22 @@
         <v>25703</v>
       </c>
       <c r="H88" t="n">
-        <v>3.6</v>
+        <v>3.3</v>
       </c>
       <c r="I88" t="n">
-        <v>2832</v>
+        <v>2614</v>
       </c>
       <c r="J88" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K88" t="n">
-        <v>0</v>
+        <v>436</v>
       </c>
       <c r="L88" t="n">
-        <v>35.8</v>
+        <v>36.1</v>
       </c>
       <c r="M88" t="n">
-        <v>28535</v>
+        <v>28753</v>
       </c>
       <c r="N88" t="inlineStr">
         <is>
@@ -4546,10 +4490,10 @@
         <v>96867</v>
       </c>
       <c r="D89" t="n">
-        <v>43.5</v>
+        <v>42.6</v>
       </c>
       <c r="E89" t="n">
-        <v>42098</v>
+        <v>41281</v>
       </c>
       <c r="F89" t="n">
         <v>48.5</v>
@@ -4558,22 +4502,22 @@
         <v>47003</v>
       </c>
       <c r="H89" t="n">
-        <v>8</v>
+        <v>7.6</v>
       </c>
       <c r="I89" t="n">
-        <v>7766</v>
+        <v>7357</v>
       </c>
       <c r="J89" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="K89" t="n">
-        <v>0</v>
+        <v>1226</v>
       </c>
       <c r="L89" t="n">
-        <v>56.5</v>
+        <v>57.4</v>
       </c>
       <c r="M89" t="n">
-        <v>54769</v>
+        <v>55586</v>
       </c>
       <c r="N89" t="inlineStr">
         <is>
@@ -4635,12 +4579,8 @@
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr"/>
-      <c r="J91" t="n">
-        <v>0</v>
-      </c>
-      <c r="K91" t="n">
-        <v>0</v>
-      </c>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr"/>
       <c r="N91" t="inlineStr">
@@ -4762,16 +4702,16 @@
         <v>6143</v>
       </c>
       <c r="H2" t="n">
-        <v>11.4</v>
+        <v>11</v>
       </c>
       <c r="I2" t="n">
-        <v>1617</v>
+        <v>1552</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="L2" t="n">
         <v>54.8</v>
@@ -4805,12 +4745,8 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
@@ -4834,10 +4770,10 @@
         <v>50210</v>
       </c>
       <c r="D4" t="n">
-        <v>61.9</v>
+        <v>61.6</v>
       </c>
       <c r="E4" t="n">
-        <v>31099</v>
+        <v>30925</v>
       </c>
       <c r="F4" t="n">
         <v>37.7</v>
@@ -4852,16 +4788,16 @@
         <v>174</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>174</v>
       </c>
       <c r="L4" t="n">
-        <v>38.1</v>
+        <v>38.4</v>
       </c>
       <c r="M4" t="n">
-        <v>19111</v>
+        <v>19285</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -5134,10 +5070,10 @@
         <v>4309</v>
       </c>
       <c r="D10" t="n">
-        <v>36.5</v>
+        <v>35.6</v>
       </c>
       <c r="E10" t="n">
-        <v>1574</v>
+        <v>1533</v>
       </c>
       <c r="F10" t="n">
         <v>54.8</v>
@@ -5146,22 +5082,22 @@
         <v>2362</v>
       </c>
       <c r="H10" t="n">
-        <v>8.699999999999999</v>
+        <v>6.7</v>
       </c>
       <c r="I10" t="n">
-        <v>373</v>
+        <v>290</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>2.9</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>124</v>
       </c>
       <c r="L10" t="n">
-        <v>63.5</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="M10" t="n">
-        <v>2735</v>
+        <v>2776</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -5246,16 +5182,16 @@
         <v>326</v>
       </c>
       <c r="H12" t="n">
-        <v>21.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>92</v>
+        <v>38</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>12.6</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="L12" t="n">
         <v>97.09999999999999</v>
@@ -5284,10 +5220,10 @@
         <v>39813</v>
       </c>
       <c r="D13" t="n">
-        <v>27.1</v>
+        <v>26.1</v>
       </c>
       <c r="E13" t="n">
-        <v>10787</v>
+        <v>10395</v>
       </c>
       <c r="F13" t="n">
         <v>66.5</v>
@@ -5296,22 +5232,22 @@
         <v>26477</v>
       </c>
       <c r="H13" t="n">
-        <v>6.4</v>
+        <v>4.4</v>
       </c>
       <c r="I13" t="n">
-        <v>2550</v>
+        <v>1765</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>1177</v>
       </c>
       <c r="L13" t="n">
-        <v>72.90000000000001</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="M13" t="n">
-        <v>29026</v>
+        <v>29418</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -5334,34 +5270,34 @@
         <v>6758</v>
       </c>
       <c r="D14" t="n">
-        <v>27.7</v>
+        <v>26.4</v>
       </c>
       <c r="E14" t="n">
-        <v>1872</v>
+        <v>1781</v>
       </c>
       <c r="F14" t="n">
-        <v>56.8</v>
+        <v>56.4</v>
       </c>
       <c r="G14" t="n">
-        <v>3836</v>
+        <v>3813</v>
       </c>
       <c r="H14" t="n">
-        <v>15.5</v>
+        <v>15.2</v>
       </c>
       <c r="I14" t="n">
-        <v>1050</v>
+        <v>1027</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>137</v>
       </c>
       <c r="L14" t="n">
-        <v>72.3</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="M14" t="n">
-        <v>4886</v>
+        <v>4977</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -5434,10 +5370,10 @@
         <v>45076</v>
       </c>
       <c r="D16" t="n">
-        <v>34.5</v>
+        <v>33.5</v>
       </c>
       <c r="E16" t="n">
-        <v>15551</v>
+        <v>15100</v>
       </c>
       <c r="F16" t="n">
         <v>51.5</v>
@@ -5446,22 +5382,22 @@
         <v>23214</v>
       </c>
       <c r="H16" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I16" t="n">
-        <v>6311</v>
+        <v>3155</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>3606</v>
       </c>
       <c r="L16" t="n">
-        <v>65.5</v>
+        <v>66.5</v>
       </c>
       <c r="M16" t="n">
-        <v>29525</v>
+        <v>29976</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -5622,34 +5558,34 @@
         <v>14588</v>
       </c>
       <c r="D20" t="n">
-        <v>26</v>
+        <v>25.6</v>
       </c>
       <c r="E20" t="n">
-        <v>3787</v>
+        <v>3741</v>
       </c>
       <c r="F20" t="n">
-        <v>63.1</v>
+        <v>62.8</v>
       </c>
       <c r="G20" t="n">
-        <v>9211</v>
+        <v>9164</v>
       </c>
       <c r="H20" t="n">
-        <v>10.3</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>1496</v>
+        <v>1262</v>
       </c>
       <c r="J20" t="n">
-        <v>0.6</v>
+        <v>2.9</v>
       </c>
       <c r="K20" t="n">
-        <v>94</v>
+        <v>421</v>
       </c>
       <c r="L20" t="n">
-        <v>74</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="M20" t="n">
-        <v>10801</v>
+        <v>10847</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -5672,10 +5608,10 @@
         <v>3188</v>
       </c>
       <c r="D21" t="n">
-        <v>47.2</v>
+        <v>46.3</v>
       </c>
       <c r="E21" t="n">
-        <v>1505</v>
+        <v>1475</v>
       </c>
       <c r="F21" t="n">
         <v>49.1</v>
@@ -5684,22 +5620,22 @@
         <v>1566</v>
       </c>
       <c r="H21" t="n">
-        <v>3.7</v>
+        <v>3.4</v>
       </c>
       <c r="I21" t="n">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="L21" t="n">
-        <v>52.8</v>
+        <v>53.7</v>
       </c>
       <c r="M21" t="n">
-        <v>1683</v>
+        <v>1713</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -5776,16 +5712,16 @@
         <v>18363</v>
       </c>
       <c r="H23" t="n">
-        <v>4.3</v>
+        <v>2.6</v>
       </c>
       <c r="I23" t="n">
-        <v>853</v>
+        <v>525</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>328</v>
       </c>
       <c r="L23" t="n">
         <v>96.7</v>
@@ -5819,12 +5755,8 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
@@ -5860,16 +5792,16 @@
         <v>1047</v>
       </c>
       <c r="H25" t="n">
-        <v>25.4</v>
+        <v>3.4</v>
       </c>
       <c r="I25" t="n">
-        <v>365</v>
+        <v>49</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>316</v>
       </c>
       <c r="L25" t="n">
         <v>98.3</v>
@@ -5879,7 +5811,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -5910,16 +5842,16 @@
         <v>14487</v>
       </c>
       <c r="H26" t="n">
-        <v>16.9</v>
+        <v>15.7</v>
       </c>
       <c r="I26" t="n">
-        <v>3642</v>
+        <v>3399</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>243</v>
       </c>
       <c r="L26" t="n">
         <v>83.90000000000001</v>
@@ -5953,12 +5885,8 @@
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" t="n">
-        <v>0</v>
-      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
@@ -5982,10 +5910,10 @@
         <v>218656</v>
       </c>
       <c r="D28" t="n">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="E28" t="n">
-        <v>15387</v>
+        <v>14577</v>
       </c>
       <c r="F28" t="n">
         <v>86.7</v>
@@ -5994,22 +5922,22 @@
         <v>189502</v>
       </c>
       <c r="H28" t="n">
-        <v>6.3</v>
+        <v>5.2</v>
       </c>
       <c r="I28" t="n">
-        <v>13767</v>
+        <v>11338</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>3239</v>
       </c>
       <c r="L28" t="n">
-        <v>93</v>
+        <v>93.3</v>
       </c>
       <c r="M28" t="n">
-        <v>203269</v>
+        <v>204079</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
@@ -6094,16 +6022,16 @@
         <v>6818</v>
       </c>
       <c r="H30" t="n">
-        <v>4.1</v>
+        <v>0.8</v>
       </c>
       <c r="I30" t="n">
-        <v>298</v>
+        <v>60</v>
       </c>
       <c r="J30" t="n">
-        <v>0</v>
+        <v>3.3</v>
       </c>
       <c r="K30" t="n">
-        <v>0</v>
+        <v>238</v>
       </c>
       <c r="L30" t="n">
         <v>98</v>
@@ -6194,16 +6122,16 @@
         <v>2679</v>
       </c>
       <c r="H32" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="I32" t="n">
-        <v>139</v>
+        <v>92</v>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K32" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="L32" t="n">
         <v>35.7</v>
@@ -6244,16 +6172,16 @@
         <v>1477</v>
       </c>
       <c r="H33" t="n">
-        <v>19.3</v>
+        <v>17.6</v>
       </c>
       <c r="I33" t="n">
-        <v>373</v>
+        <v>341</v>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="K33" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="L33" t="n">
         <v>95.8</v>
@@ -6294,16 +6222,16 @@
         <v>177715</v>
       </c>
       <c r="H34" t="n">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="I34" t="n">
-        <v>3332</v>
+        <v>2221</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>1111</v>
       </c>
       <c r="L34" t="n">
         <v>84.5</v>
@@ -6444,16 +6372,16 @@
         <v>15009</v>
       </c>
       <c r="H37" t="n">
-        <v>2.1</v>
+        <v>0.8</v>
       </c>
       <c r="I37" t="n">
-        <v>419</v>
+        <v>168</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="K37" t="n">
-        <v>0</v>
+        <v>252</v>
       </c>
       <c r="L37" t="n">
         <v>76</v>
@@ -6482,34 +6410,34 @@
         <v>21382</v>
       </c>
       <c r="D38" t="n">
-        <v>21.6</v>
+        <v>20.9</v>
       </c>
       <c r="E38" t="n">
-        <v>4627</v>
+        <v>4468</v>
       </c>
       <c r="F38" t="n">
-        <v>75</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="G38" t="n">
-        <v>16037</v>
+        <v>15957</v>
       </c>
       <c r="H38" t="n">
-        <v>3.4</v>
+        <v>1.9</v>
       </c>
       <c r="I38" t="n">
-        <v>718</v>
+        <v>399</v>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>2.6</v>
       </c>
       <c r="K38" t="n">
-        <v>0</v>
+        <v>558</v>
       </c>
       <c r="L38" t="n">
-        <v>78.40000000000001</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>16755</v>
+        <v>16914</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
@@ -6544,16 +6472,16 @@
         <v>1439</v>
       </c>
       <c r="H39" t="n">
-        <v>15.2</v>
+        <v>13.9</v>
       </c>
       <c r="I39" t="n">
-        <v>411</v>
+        <v>377</v>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="K39" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="L39" t="n">
         <v>68.40000000000001</v>
@@ -6582,10 +6510,10 @@
         <v>4578</v>
       </c>
       <c r="D40" t="n">
-        <v>18.6</v>
+        <v>18.3</v>
       </c>
       <c r="E40" t="n">
-        <v>851</v>
+        <v>838</v>
       </c>
       <c r="F40" t="n">
         <v>72.40000000000001</v>
@@ -6594,22 +6522,22 @@
         <v>3314</v>
       </c>
       <c r="H40" t="n">
-        <v>9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I40" t="n">
-        <v>413</v>
+        <v>374</v>
       </c>
       <c r="J40" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="K40" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="L40" t="n">
-        <v>81.40000000000001</v>
+        <v>81.7</v>
       </c>
       <c r="M40" t="n">
-        <v>3727</v>
+        <v>3740</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
@@ -6632,10 +6560,10 @@
         <v>3680</v>
       </c>
       <c r="D41" t="n">
-        <v>59</v>
+        <v>58.7</v>
       </c>
       <c r="E41" t="n">
-        <v>2170</v>
+        <v>2158</v>
       </c>
       <c r="F41" t="n">
         <v>32.7</v>
@@ -6650,16 +6578,16 @@
         <v>307</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="K41" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="L41" t="n">
-        <v>41</v>
+        <v>41.3</v>
       </c>
       <c r="M41" t="n">
-        <v>1510</v>
+        <v>1522</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
@@ -6682,16 +6610,16 @@
         <v>34813</v>
       </c>
       <c r="D42" t="n">
-        <v>17.5</v>
+        <v>17</v>
       </c>
       <c r="E42" t="n">
-        <v>6076</v>
+        <v>5912</v>
       </c>
       <c r="F42" t="n">
-        <v>78.3</v>
+        <v>77.8</v>
       </c>
       <c r="G42" t="n">
-        <v>27259</v>
+        <v>27095</v>
       </c>
       <c r="H42" t="n">
         <v>3.8</v>
@@ -6700,16 +6628,16 @@
         <v>1314</v>
       </c>
       <c r="J42" t="n">
-        <v>0.5</v>
+        <v>1.4</v>
       </c>
       <c r="K42" t="n">
-        <v>164</v>
+        <v>493</v>
       </c>
       <c r="L42" t="n">
-        <v>82.5</v>
+        <v>83</v>
       </c>
       <c r="M42" t="n">
-        <v>28737</v>
+        <v>28901</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
@@ -6786,16 +6714,16 @@
         <v>5029</v>
       </c>
       <c r="H44" t="n">
-        <v>2.8</v>
+        <v>2</v>
       </c>
       <c r="I44" t="n">
-        <v>157</v>
+        <v>112</v>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="K44" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="L44" t="n">
         <v>92.8</v>
@@ -6824,10 +6752,10 @@
         <v>55127</v>
       </c>
       <c r="D45" t="n">
-        <v>65.40000000000001</v>
+        <v>63.6</v>
       </c>
       <c r="E45" t="n">
-        <v>36074</v>
+        <v>35058</v>
       </c>
       <c r="F45" t="n">
         <v>14.3</v>
@@ -6836,22 +6764,22 @@
         <v>7875</v>
       </c>
       <c r="H45" t="n">
-        <v>19.8</v>
+        <v>13.8</v>
       </c>
       <c r="I45" t="n">
-        <v>10924</v>
+        <v>7621</v>
       </c>
       <c r="J45" t="n">
-        <v>0.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="K45" t="n">
-        <v>254</v>
+        <v>4573</v>
       </c>
       <c r="L45" t="n">
-        <v>34.6</v>
+        <v>36.4</v>
       </c>
       <c r="M45" t="n">
-        <v>19053</v>
+        <v>20069</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
@@ -6874,10 +6802,10 @@
         <v>25164</v>
       </c>
       <c r="D46" t="n">
-        <v>37.5</v>
+        <v>36.8</v>
       </c>
       <c r="E46" t="n">
-        <v>9449</v>
+        <v>9250</v>
       </c>
       <c r="F46" t="n">
         <v>56.9</v>
@@ -6886,22 +6814,22 @@
         <v>14323</v>
       </c>
       <c r="H46" t="n">
-        <v>5.5</v>
+        <v>4.7</v>
       </c>
       <c r="I46" t="n">
-        <v>1392</v>
+        <v>1194</v>
       </c>
       <c r="J46" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="K46" t="n">
-        <v>0</v>
+        <v>398</v>
       </c>
       <c r="L46" t="n">
-        <v>62.5</v>
+        <v>63.2</v>
       </c>
       <c r="M46" t="n">
-        <v>15715</v>
+        <v>15914</v>
       </c>
       <c r="N46" t="inlineStr">
         <is>
@@ -6957,14 +6885,14 @@
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="n">
-        <v>0</v>
-      </c>
-      <c r="K48" t="n">
-        <v>0</v>
-      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr">
@@ -7000,16 +6928,16 @@
         <v>57687</v>
       </c>
       <c r="H49" t="n">
-        <v>2.3</v>
+        <v>1.9</v>
       </c>
       <c r="I49" t="n">
-        <v>1822</v>
+        <v>1518</v>
       </c>
       <c r="J49" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="K49" t="n">
-        <v>0</v>
+        <v>304</v>
       </c>
       <c r="L49" t="n">
         <v>73.7</v>
@@ -7097,12 +7025,8 @@
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr"/>
-      <c r="J51" t="n">
-        <v>0</v>
-      </c>
-      <c r="K51" t="n">
-        <v>0</v>
-      </c>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr">

</xml_diff>